<commit_message>
Correcting typos in key
</commit_message>
<xml_diff>
--- a/Plates/nitrite_key.xlsx
+++ b/Plates/nitrite_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaedonswanson/Desktop/School/MS/Research/Microplate/Plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B24F2401-53DC-E149-8752-59CEE25ED7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D03FFF-7262-304A-A9A6-1C81582D0961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="6" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="3" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Format" sheetId="1" r:id="rId1"/>
@@ -158,9 +158,6 @@
     <t>adams-mid-up_06192026</t>
   </si>
   <si>
-    <t>elm-bridge-06192026</t>
-  </si>
-  <si>
     <t>adams-mid-down_06192026</t>
   </si>
   <si>
@@ -176,9 +173,6 @@
     <t>heron-map_06192026</t>
   </si>
   <si>
-    <t>gcp-06192026</t>
-  </si>
-  <si>
     <t>elm-bridge_06212026</t>
   </si>
   <si>
@@ -267,6 +261,12 @@
   </si>
   <si>
     <t>heron-resi_08052026</t>
+  </si>
+  <si>
+    <t>elm-bridge_06192026</t>
+  </si>
+  <si>
+    <t>gcp_06192026</t>
   </si>
 </sst>
 </file>
@@ -1491,13 +1491,13 @@
         <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="J3" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -1514,13 +1514,13 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1537,13 +1537,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1560,13 +1560,13 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1583,13 +1583,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1606,13 +1606,13 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1629,13 +1629,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1048576" spans="5:7" x14ac:dyDescent="0.2">
@@ -1715,22 +1715,22 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -1747,22 +1747,22 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -1779,13 +1779,13 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1802,13 +1802,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1825,13 +1825,13 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1848,13 +1848,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1871,13 +1871,13 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1894,13 +1894,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1970,31 +1970,31 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="K2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -2011,31 +2011,31 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="K3" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -2052,31 +2052,31 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -2093,31 +2093,31 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -2134,22 +2134,22 @@
         <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -2166,22 +2166,22 @@
         <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -2198,22 +2198,22 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -2230,22 +2230,22 @@
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2315,22 +2315,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2350,22 +2350,22 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2385,16 +2385,16 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -2416,16 +2416,16 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
@@ -2447,16 +2447,16 @@
         <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -2475,16 +2475,16 @@
         <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -2503,16 +2503,16 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -2531,16 +2531,16 @@
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -2551,6 +2551,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2559,7 +2565,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F4F88F6F7EE4CD4B82C1B33855E0F7E8" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="64cb4cc7036794b82b9e5aa8e91c3622">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399018e3-b857-408b-bd21-a6a80c979a4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94968af49f0175a612c20130cdc28d5d" ns2:_="">
     <xsd:import namespace="399018e3-b857-408b-bd21-a6a80c979a4e"/>
@@ -2697,13 +2703,23 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A12E62EB-4C13-40F4-82AA-4D1604D83A1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EE035F8-D68E-4C69-8A9A-AC5006D01AC3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2711,7 +2727,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF451231-11C1-40DC-B808-D626057CF16F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2727,20 +2743,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A12E62EB-4C13-40F4-82AA-4D1604D83A1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updating incorrect date format(s)
</commit_message>
<xml_diff>
--- a/Plates/nitrite_key.xlsx
+++ b/Plates/nitrite_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaedonswanson/Desktop/School/MS/Research/Microplate/Plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D03FFF-7262-304A-A9A6-1C81582D0961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FAE9C2-4773-514B-9192-C4A69921BE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="3" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Format" sheetId="1" r:id="rId1"/>
@@ -122,33 +122,6 @@
     <t>elm-school_06122026</t>
   </si>
   <si>
-    <t>her-map_20260617</t>
-  </si>
-  <si>
-    <t>gcp_20260617</t>
-  </si>
-  <si>
-    <t>her-resi_20260617</t>
-  </si>
-  <si>
-    <t>her-out_20260617</t>
-  </si>
-  <si>
-    <t>elm-school_20260617</t>
-  </si>
-  <si>
-    <t>elm-bridge_20260617</t>
-  </si>
-  <si>
-    <t>adams-in_20260617</t>
-  </si>
-  <si>
-    <t>adams-mid_20260617</t>
-  </si>
-  <si>
-    <t>adams-out_20260617</t>
-  </si>
-  <si>
     <t>adams-out_06192026</t>
   </si>
   <si>
@@ -267,6 +240,33 @@
   </si>
   <si>
     <t>gcp_06192026</t>
+  </si>
+  <si>
+    <t>gcp_06172026</t>
+  </si>
+  <si>
+    <t>her-map_06172026</t>
+  </si>
+  <si>
+    <t>her-out_06172026</t>
+  </si>
+  <si>
+    <t>elm-school_06172026</t>
+  </si>
+  <si>
+    <t>elm-bridge_06172026</t>
+  </si>
+  <si>
+    <t>adams-in_06172026</t>
+  </si>
+  <si>
+    <t>adams-mid_06172026</t>
+  </si>
+  <si>
+    <t>adams-out_06172026</t>
+  </si>
+  <si>
+    <t>her-resi_06172026</t>
   </si>
 </sst>
 </file>
@@ -854,6 +854,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="K6:M6"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E2:G2"/>
@@ -870,22 +886,6 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K8:M8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1202,22 +1202,22 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="J2" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1234,13 +1234,13 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1257,13 +1257,13 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1280,13 +1280,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1303,13 +1303,13 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1326,13 +1326,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1349,13 +1349,13 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1372,13 +1372,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1450,22 +1450,22 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="I2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="J2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -1482,22 +1482,22 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="J3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -1514,13 +1514,13 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1537,13 +1537,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1560,13 +1560,13 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1583,13 +1583,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1606,13 +1606,13 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1629,13 +1629,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1048576" spans="5:7" x14ac:dyDescent="0.2">
@@ -1715,22 +1715,22 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="I2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -1747,22 +1747,22 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -1779,13 +1779,13 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1802,13 +1802,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1825,13 +1825,13 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1848,13 +1848,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1871,13 +1871,13 @@
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1894,13 +1894,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1970,31 +1970,31 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -2011,31 +2011,31 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -2052,31 +2052,31 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -2093,31 +2093,31 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -2134,22 +2134,22 @@
         <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -2166,22 +2166,22 @@
         <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -2198,22 +2198,22 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -2230,22 +2230,22 @@
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2315,22 +2315,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2350,22 +2350,22 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2385,16 +2385,16 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -2416,16 +2416,16 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
@@ -2447,16 +2447,16 @@
         <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -2475,16 +2475,16 @@
         <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -2503,16 +2503,16 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -2531,16 +2531,16 @@
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -2551,21 +2551,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F4F88F6F7EE4CD4B82C1B33855E0F7E8" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="64cb4cc7036794b82b9e5aa8e91c3622">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399018e3-b857-408b-bd21-a6a80c979a4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94968af49f0175a612c20130cdc28d5d" ns2:_="">
     <xsd:import namespace="399018e3-b857-408b-bd21-a6a80c979a4e"/>
@@ -2703,31 +2688,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A12E62EB-4C13-40F4-82AA-4D1604D83A1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EE035F8-D68E-4C69-8A9A-AC5006D01AC3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF451231-11C1-40DC-B808-D626057CF16F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2743,4 +2719,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EE035F8-D68E-4C69-8A9A-AC5006D01AC3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A12E62EB-4C13-40F4-82AA-4D1604D83A1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>